<commit_message>
feat(F-NAR-019): TREE-COL-007 polish La porte embuée et les bottes de Nino
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-007.xlsx
+++ b/stories/arbres/TREE-COL-007.xlsx
@@ -4645,17 +4645,17 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes et le crayon dorment dans la lumière.</t>
+          <t>Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes, le crayon et un croissant de buée dorment dans la lumière.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes et le crayon dorment dans la lumière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes, le crayon et un croissant de buée dorment dans la lumière.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes et le crayon dorment dans la lumière. [pause]</t>
+          <t>Le soir, le crayon de poche dépasse du manteau. Papa range les chaussures, le dos tourné. Regarde mes virgules ! Papa entend le mot virgules, pas le reste. Nino s'assoit, le crayon en l'air. Il attend qu'il se tourne. Je te vois. Montre-moi. À l'école, j'ai tracé les bottes, après l'attente. Papa pose le crayon à côté, sans le prendre. Le rond de la lampe est assez grand pour deux. Les bottes, le crayon et un croissant de buée dorment dans la lumière. [pause]</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -4800,7 +4800,7 @@
 enfant-m|À l'école, j'ai tracé les bottes, après l'attente.
 narrateur|Papa pose le crayon à côté, sans le prendre.
 maman|Le rond de la lampe est assez grand pour deux.
-narrateur|Les bottes et le crayon dorment dans la lumière.</t>
+narrateur|Les bottes, le crayon et un croissant de buée dorment dans la lumière.</t>
         </is>
       </c>
       <c r="AX20" t="inlineStr">
@@ -6163,17 +6163,17 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent, comme un petit tambour. On les pose près du radiateur, sur le dernier mot.</t>
+          <t>Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent. Un croissant de buée suit le rythme. On les pose près du radiateur, sur le dernier mot.</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent, comme un petit tambour. On les pose près du radiateur, sur le dernier mot.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent. Un croissant de buée suit le rythme. On les pose près du radiateur, sur le dernier mot.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent, comme un petit tambour. On les pose près du radiateur, sur le dernier mot. [pause]</t>
+          <t>Le soir, papa chante en rangeant le manteau. Bottes, bottes ! Les deux voix se marchent dessus, près du tapis. Laisse-moi finir. Ensuite, ton couplet. Nino attend, un pied sur la laine. À l'école, j'ai trop chanté tôt. Le fil a cassé. Papa s'arrête pile, et penche l'oreille. Bottes, bottes, sur le tapis. Cette fois, ta note a toute la place. Les boucles vibrent. Un croissant de buée suit le rythme. On les pose près du radiateur, sur le dernier mot. [pause]</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -6318,7 +6318,8 @@
 narrateur|Papa s'arrête pile, et penche l'oreille.
 enfant-m|Bottes, bottes, sur le tapis.
 maman|Cette fois, ta note a toute la place.
-narrateur|Les boucles vibrent, comme un petit tambour.
+narrateur|Les boucles vibrent.
+narrateur|Un croissant de buée suit le rythme.
 papa|On les pose près du radiateur, sur le dernier mot.</t>
         </is>
       </c>
@@ -6351,17 +6352,17 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Nino a chanté les bottes, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le radiateur n'a plus de tic, plus de refrain.</t>
+          <t>Nino a chanté les bottes, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le croissant de buée quitte le radiateur, sans refrain.</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a chanté les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt;, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le radiateur n'a plus de tic, plus de refrain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a chanté les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt;, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le croissant de buée quitte le radiateur, sans refrain.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a chanté les &lt;emphasis&gt;bottes&lt;/emphasis&gt;, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le radiateur n'a plus de tic, plus de refrain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a chanté les &lt;emphasis&gt;bottes&lt;/emphasis&gt;, après le manteau. J'ai fini, puis toi. Merci d'avoir laissé le couplet de papa. Le fil n'a pas cassé, cette fois. Une note de la chanson reste dans la vapeur du cacao. Les boucles vibrent, puis s'arrêtent. Le moment où ça cassait, tu le dis ? Oui. Sur le tapis. Le croissant de buée quitte le radiateur, sans refrain.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr"/>
@@ -6508,7 +6509,7 @@
 papa|Le moment où ça cassait, tu le dis ?
 enfant-m|Oui.
 enfant-m|Sur le tapis.
-narrateur|Le radiateur n'a plus de tic, plus de refrain.</t>
+narrateur|Le croissant de buée quitte le radiateur, sans refrain.</t>
         </is>
       </c>
       <c r="AX29" t="inlineStr">
@@ -6920,17 +6921,17 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend dans le calme ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche.</t>
+          <t>Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend sans le bruit ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend dans le calme ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend sans le bruit ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend dans le calme ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche. [pause]</t>
+          <t>Nino grimpe sur la chaise, près de la table. Le bois est lisse, un peu froid. Ma phrase, tout de suite ! La chaise racle. Le bruit couvre les mots. La maîtresse lève les yeux, puis reprend. Nino se rassoit, le ventre serré. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Il pose les mains à plat, sur le bois. Il attend que la racle se taise. Je m'accroupis, près des pieds de la chaise. Ta phrase, on la prend sans le bruit ? Oui. Un camarade a parlé trop fort. Ça m'a pincé, ici. Merci d'avoir gardé tes mains sur la table. Un crayon roule, et s'arrête contre sa manche. [pause]</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
@@ -7076,7 +7077,7 @@
 narrateur|Il pose les mains à plat, sur le bois.
 narrateur|Il attend que la racle se taise.
 papa|Je m'accroupis, près des pieds de la chaise.
-maman|Ta phrase, on la prend dans le calme ?
+maman|Ta phrase, on la prend sans le bruit ?
 enfant-m|Oui.
 enfant-m|Un camarade a parlé trop fort.
 enfant-m|Ça m'a pincé, ici.
@@ -16464,17 +16465,17 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans la vapeur, et s'y perd. Cette fois, ma note a eu le silence.</t>
+          <t>Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans le croissant de vapeur, et s'y perd. Cette fois, ma note a eu le silence.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans la vapeur, et s'y perd. Cette fois, ma note a eu le silence.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans le croissant de vapeur, et s'y perd. Cette fois, ma note a eu le silence.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans la vapeur, et s'y perd. Cette fois, ma note a eu le silence. [pause]</t>
+          <t>Le soir, Nino entre avec une note du préau, trop haute. La casserole répond, trop basse. C'est ma chanson de gouttes ! La mienne, c'est le thym. Une après l'autre. Nino se tait. Une botte claque, puis plus. Sous le toit, j'ai chanté dans l'eau. Après, dans le creux. Chante-moi le creux, ici. Nino glisse sa note. La vapeur danse, sans ploc. On pose les bottes sur le dernier mot. Le couplet rentre dans le croissant de vapeur, et s'y perd. Cette fois, ma note a eu le silence. [pause]</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -16621,7 +16622,7 @@
 narrateur|Nino glisse sa note.
 narrateur|La vapeur danse, sans ploc.
 papa|On pose les bottes sur le dernier mot.
-narrateur|Le couplet rentre dans la vapeur, et s'y perd.
+narrateur|Le couplet rentre dans le croissant de vapeur, et s'y perd.
 enfant-m|Cette fois, ma note a eu le silence.</t>
         </is>
       </c>
@@ -16654,17 +16655,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les bottes attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque, puis plus.</t>
+          <t>Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les bottes attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque. Le croissant de buée s'en va.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque, puis plus.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque. Le croissant de buée s'en va.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les &lt;emphasis&gt;bottes&lt;/emphasis&gt; attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque, puis plus.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a chanté le creux, après le thym. J'ai eu ta note. Merci. Les &lt;emphasis&gt;bottes&lt;/emphasis&gt; attendent le dernier mot. Dans l'eau, puis dans le silence. Le couplet rentre dans la vapeur, et s'y perd. La casserole ne répond plus, trop basse. Tu gardes la note trop haute ? Surtout celle-là. Une botte claque. Le croissant de buée s'en va.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16811,7 +16812,8 @@
 narrateur|La casserole ne répond plus, trop basse.
 maman|Tu gardes la note trop haute ?
 enfant-m|Surtout celle-là.
-narrateur|Une botte claque, puis plus.</t>
+narrateur|Une botte claque.
+narrateur|Le croissant de buée s'en va.</t>
         </is>
       </c>
       <c r="AX83" t="inlineStr">
@@ -17224,17 +17226,17 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment, légères, près du bois.</t>
+          <t>Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment près du croissant de buée.</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment, légères, près du bois.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment près du croissant de buée.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment, légères, près du bois. [pause]</t>
+          <t>Le soir, Sarah tapote le bol, un, deux. C'est le rythme du préau ! Il chante par-dessus. Le bol tressaute. Un tap, puis l'autre. Le tien après le mien. Nino compte. Il glisse sa note dans le trou. J'ai chanté dans l'eau. Après, dans le silence. On a le silence, ici. Sarah pousse le bol. Le bonnet rouge ne goutte plus. Toi, tu as le creux. Moi, le bonnet. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment près du croissant de buée. [pause]</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -17384,7 +17386,7 @@
 enfant-f|Toi, tu as le creux.
 enfant-f|Moi, le bonnet.
 narrateur|Sarah chante tout bas, une fois, puis le bol se tait.
-narrateur|Les bottes s'endorment, légères, près du bois.</t>
+narrateur|Les bottes s'endorment près du croissant de buée.</t>
         </is>
       </c>
       <c r="AX86" t="inlineStr">
@@ -17416,17 +17418,17 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le bonnet rouge ne goutte plus, plus du tout.</t>
+          <t>Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les bottes s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le croissant de buée s'endort sur le bonnet rouge.</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le bonnet rouge ne goutte plus, plus du tout.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les &lt;emphasis level="moderate"&gt;bottes&lt;/emphasis&gt; s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le croissant de buée s'endort sur le bonnet rouge.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les &lt;emphasis&gt;bottes&lt;/emphasis&gt; s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le bonnet rouge ne goutte plus, plus du tout.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Nino a glissé sa note dans le trou de Sarah. Toi, tu as le creux. Moi, le bonnet. On a le silence, ici. Merci, les deux rythmes. Sarah chante tout bas, une fois, puis le bol se tait. Les &lt;emphasis&gt;bottes&lt;/emphasis&gt; s'endorment, légères, près du bois. J'ai chanté dans l'eau. Après, dans le silence. Moi, j'ai tapoté, puis j'ai écouté. Le croissant de buée s'endort sur le bonnet rouge.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -17574,7 +17576,7 @@
 enfant-m|J'ai chanté dans l'eau.
 enfant-m|Après, dans le silence.
 enfant-f|Moi, j'ai tapoté, puis j'ai écouté.
-narrateur|Le bonnet rouge ne goutte plus, plus du tout.</t>
+narrateur|Le croissant de buée s'endort sur le bonnet rouge.</t>
         </is>
       </c>
       <c r="AX87" t="inlineStr">
@@ -17600,7 +17602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17664,6 +17666,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>